<commit_message>
feat: Implement advanced domain expert features, data preparation, and hyperparameter optimization scripts, alongside new cache and prediction result files.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-17.xlsx
+++ b/results/nba_predictions_2025-12-17.xlsx
@@ -562,16 +562,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>52.48</v>
+        <v>43.24</v>
       </c>
       <c r="E2" t="n">
-        <v>47.52</v>
+        <v>56.76</v>
       </c>
       <c r="F2" t="n">
-        <v>54.87</v>
+        <v>54.81</v>
       </c>
       <c r="G2" t="n">
-        <v>45.13</v>
+        <v>45.19</v>
       </c>
       <c r="H2" t="n">
         <v>-0.43</v>
@@ -593,7 +593,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -607,11 +607,13 @@
       <c r="Q2" t="n">
         <v>0</v>
       </c>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="n">
-        <v>230.2</v>
-      </c>
+      <c r="R2" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="S2" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
         <is>
           <t>Ayo Dosunmu (QUESTIONABLE)</t>
@@ -623,7 +625,7 @@
         </is>
       </c>
       <c r="W2" t="n">
-        <v>1.5</v>
+        <v>-4.1</v>
       </c>
     </row>
     <row r="3">
@@ -643,16 +645,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>54.15</v>
+        <v>66.67</v>
       </c>
       <c r="E3" t="n">
-        <v>45.85</v>
+        <v>33.33</v>
       </c>
       <c r="F3" t="n">
-        <v>57.37</v>
+        <v>57.35</v>
       </c>
       <c r="G3" t="n">
-        <v>42.63</v>
+        <v>42.65</v>
       </c>
       <c r="H3" t="n">
         <v>-0.04</v>
@@ -674,7 +676,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -688,11 +690,13 @@
       <c r="Q3" t="n">
         <v>0</v>
       </c>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="n">
-        <v>219.8</v>
-      </c>
+      <c r="R3" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="S3" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
           <t>Joan Beringer (OUT)</t>
@@ -704,7 +708,7 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>2.5</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Introduce quantum props prediction pipeline with data scraper, model training, and MLflow tracking.
</commit_message>
<xml_diff>
--- a/results/nba_predictions_2025-12-17.xlsx
+++ b/results/nba_predictions_2025-12-17.xlsx
@@ -568,10 +568,10 @@
         <v>56.76</v>
       </c>
       <c r="F2" t="n">
-        <v>54.81</v>
+        <v>54.86</v>
       </c>
       <c r="G2" t="n">
-        <v>45.19</v>
+        <v>45.14</v>
       </c>
       <c r="H2" t="n">
         <v>-0.43</v>
@@ -651,10 +651,10 @@
         <v>33.33</v>
       </c>
       <c r="F3" t="n">
-        <v>57.35</v>
+        <v>57.4</v>
       </c>
       <c r="G3" t="n">
-        <v>42.65</v>
+        <v>42.6</v>
       </c>
       <c r="H3" t="n">
         <v>-0.04</v>

</xml_diff>